<commit_message>
Model v36: terminal growth and refinancing rate as inputs
- Terminal growth moved to Inputs D124; the DCF summary and the
  sensitivity table centre both link to it, so the base valuation and
  football field follow a change in terminal growth.
- Pre-tax cost of debt (Inputs D119) is now an input and also sets the
  bank loan rate after the June 2028 refinancing.
- Values unchanged: base CZK 460, upside 633 / 654, downside 180 / 310.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CmjhbXW2V6KhqYE6XGCFnf
</commit_message>
<xml_diff>
--- a/Balko_Kofola_Valuation_Model.xlsx
+++ b/Balko_Kofola_Valuation_Model.xlsx
@@ -37,7 +37,7 @@
     <definedName name="ValDate">Inputs!$D$11</definedName>
     <definedName name="WACC">Outputs!$D$8</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1499" uniqueCount="751">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1502" uniqueCount="751">
   <si>
     <t>Kofola ČeskoSlovensko  |  Model</t>
   </si>
@@ -852,7 +852,7 @@
     <t>NCI share of net profit</t>
   </si>
   <si>
-    <t>WACC build</t>
+    <t>WACC and terminal growth</t>
   </si>
   <si>
     <t>Risk-free rate</t>
@@ -885,7 +885,7 @@
     <t>Cost of equity</t>
   </si>
   <si>
-    <t>Pre-tax cost of debt</t>
+    <t>Pre-tax cost of debt (refinancing rate from 2028)</t>
   </si>
   <si>
     <t>After-tax cost of debt</t>
@@ -14035,7 +14035,8 @@
       <c r="B9" s="8" t="s">
         <v>169</v>
       </c>
-      <c r="D9" s="121">
+      <c r="D9" s="120">
+        <f>Inputs!D124</f>
         <v>0.02</v>
       </c>
       <c r="N9" s="122" t="s">
@@ -15648,7 +15649,8 @@
         <f>G107-$D$102</f>
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="G107" s="176">
+      <c r="G107" s="175">
+        <f>Inputs!$D$124</f>
         <v>0.02</v>
       </c>
       <c r="H107" s="175">
@@ -18888,13 +18890,16 @@
       <c r="I87" s="104">
         <v>0.05</v>
       </c>
-      <c r="J87" s="104">
+      <c r="J87" s="95">
+        <f>$D$119</f>
         <v>0.05</v>
       </c>
-      <c r="K87" s="104">
+      <c r="K87" s="95">
+        <f>$D$119</f>
         <v>0.05</v>
       </c>
-      <c r="L87" s="104">
+      <c r="L87" s="95">
+        <f>$D$119</f>
         <v>0.05</v>
       </c>
       <c r="M87" s="78"/>
@@ -19502,8 +19507,7 @@
       <c r="C119" s="124" t="s">
         <v>194</v>
       </c>
-      <c r="D119" s="128">
-        <f>H87</f>
+      <c r="D119" s="125">
         <v>0.05</v>
       </c>
       <c r="E119" s="134"/>
@@ -19589,6 +19593,20 @@
       </c>
       <c r="E123" s="126"/>
       <c r="N123" s="127"/>
+    </row>
+    <row r="124" spans="1:14" outlineLevel="1" x14ac:dyDescent="0.15">
+      <c r="B124" s="123" t="s">
+        <v>169</v>
+      </c>
+      <c r="C124" s="124" t="s">
+        <v>194</v>
+      </c>
+      <c r="D124" s="125">
+        <v>0.02</v>
+      </c>
+      <c r="N124" s="124" t="s">
+        <v>655</v>
+      </c>
     </row>
     <row r="125" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A125" s="107"/>

</xml_diff>